<commit_message>
Add betting advisor to streamlit
</commit_message>
<xml_diff>
--- a/data/passing-prop-predictions-2025.xlsx
+++ b/data/passing-prop-predictions-2025.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/98038a0616e2a1bf/Desktop/Development/Projects/nfl-prop-model-2/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_04E55082DCEDC07E2FDAD079445BB426E960B561" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{324E5CDE-CF0A-4F50-9E2E-CAFDAF0F1BB4}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="11_2BDDA100C818C55DB68CC132954B5956B0404189" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4152FBA0-E3D6-4271-A9D8-F3D4EC37FA82}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10260" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10260" firstSheet="2" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Week 1" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1237" uniqueCount="280">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1333" uniqueCount="285">
   <si>
     <t>Player</t>
   </si>
@@ -865,14 +865,29 @@
     <t>58.5%</t>
   </si>
   <si>
-    <t>40.7%</t>
+    <t>55.4%</t>
+  </si>
+  <si>
+    <t>57.8%</t>
+  </si>
+  <si>
+    <t>58.0%</t>
+  </si>
+  <si>
+    <t>56.5%</t>
+  </si>
+  <si>
+    <t>58.8%</t>
+  </si>
+  <si>
+    <t>61.4%</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -896,8 +911,13 @@
       <color theme="1"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -940,6 +960,36 @@
         <bgColor rgb="FF90EE90"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF90EE90"/>
+        <bgColor rgb="FF90EE90"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF90EE90"/>
+        <bgColor rgb="FF90EE90"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF90EE90"/>
+        <bgColor rgb="FF90EE90"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF90EE90"/>
+        <bgColor rgb="FF90EE90"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF90EE90"/>
+        <bgColor rgb="FF90EE90"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -953,7 +1003,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -996,6 +1046,24 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1222,7 +1290,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-468D-4FDC-8D47-23D4A658F5FA}"/>
+              <c16:uniqueId val="{00000000-0F74-479D-8B89-D2F319169077}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1401,7 +1469,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-468D-4FDC-8D47-23D4A658F5FA}"/>
+              <c16:uniqueId val="{00000001-0F74-479D-8B89-D2F319169077}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -38842,59 +38910,60 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:M19"/>
   <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="1" max="1" width="11" customWidth="1"/>
+    <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="6" customWidth="1"/>
     <col min="3" max="3" width="10" customWidth="1"/>
-    <col min="4" max="5" width="11" customWidth="1"/>
+    <col min="4" max="4" width="11" customWidth="1"/>
+    <col min="5" max="5" width="20" customWidth="1"/>
     <col min="6" max="6" width="12" customWidth="1"/>
     <col min="7" max="7" width="8" customWidth="1"/>
     <col min="8" max="8" width="11" customWidth="1"/>
     <col min="9" max="9" width="7" customWidth="1"/>
-    <col min="10" max="10" width="6" customWidth="1"/>
+    <col min="10" max="10" width="10" customWidth="1"/>
     <col min="11" max="13" width="7" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.75">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="20" t="s">
         <v>12</v>
       </c>
     </row>
@@ -38919,20 +38988,20 @@
       </c>
       <c r="G2" s="13"/>
       <c r="H2" s="13" t="s">
-        <v>279</v>
+        <v>220</v>
       </c>
       <c r="I2" s="14" t="s">
         <v>26</v>
       </c>
       <c r="J2" s="13"/>
       <c r="K2" s="13">
-        <v>142.6</v>
+        <v>143.19999999999999</v>
       </c>
       <c r="L2" s="13">
-        <v>219.1</v>
+        <v>218</v>
       </c>
       <c r="M2" s="13">
-        <v>294</v>
+        <v>293.7</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.75">
@@ -38956,36 +39025,613 @@
       </c>
       <c r="G3" s="13"/>
       <c r="H3" s="13" t="s">
-        <v>83</v>
+        <v>279</v>
       </c>
       <c r="I3" s="15" t="s">
         <v>19</v>
       </c>
       <c r="J3" s="13"/>
       <c r="K3" s="13">
-        <v>150.1</v>
+        <v>150.6</v>
       </c>
       <c r="L3" s="13">
-        <v>224.5</v>
+        <v>224.1</v>
       </c>
       <c r="M3" s="13">
-        <v>300.3</v>
+        <v>297.60000000000002</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.75">
-      <c r="A4" s="13"/>
-      <c r="B4" s="13"/>
-      <c r="C4" s="13"/>
-      <c r="D4" s="13"/>
-      <c r="E4" s="13"/>
-      <c r="F4" s="13"/>
+      <c r="A4" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="B4" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="E4" s="13">
+        <v>261.39999389648438</v>
+      </c>
+      <c r="F4" s="13">
+        <v>250.5</v>
+      </c>
       <c r="G4" s="13"/>
-      <c r="H4" s="13"/>
-      <c r="I4" s="13"/>
+      <c r="H4" s="13" t="s">
+        <v>280</v>
+      </c>
+      <c r="I4" s="15" t="s">
+        <v>19</v>
+      </c>
       <c r="J4" s="13"/>
-      <c r="K4" s="13"/>
-      <c r="L4" s="13"/>
-      <c r="M4" s="13"/>
+      <c r="K4" s="13">
+        <v>186.4</v>
+      </c>
+      <c r="L4" s="13">
+        <v>262.10000000000002</v>
+      </c>
+      <c r="M4" s="13">
+        <v>337.1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.75">
+      <c r="A5" s="13" t="s">
+        <v>49</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="E5" s="13">
+        <v>234.30000305175781</v>
+      </c>
+      <c r="F5" s="13">
+        <v>222.5</v>
+      </c>
+      <c r="G5" s="13"/>
+      <c r="H5" s="13" t="s">
+        <v>281</v>
+      </c>
+      <c r="I5" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="J5" s="13"/>
+      <c r="K5" s="13">
+        <v>158</v>
+      </c>
+      <c r="L5" s="13">
+        <v>233.9</v>
+      </c>
+      <c r="M5" s="13">
+        <v>311.39999999999998</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.75">
+      <c r="A6" s="13" t="s">
+        <v>114</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>115</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="D6" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" s="13">
+        <v>233.69999694824219</v>
+      </c>
+      <c r="F6" s="13">
+        <v>218.5</v>
+      </c>
+      <c r="G6" s="13"/>
+      <c r="H6" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="I6" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="J6" s="13"/>
+      <c r="K6" s="13">
+        <v>158.69999999999999</v>
+      </c>
+      <c r="L6" s="13">
+        <v>233</v>
+      </c>
+      <c r="M6" s="13">
+        <v>308.2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.75">
+      <c r="A7" s="13" t="s">
+        <v>81</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="D7" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="E7" s="13">
+        <v>222.6000061035156</v>
+      </c>
+      <c r="F7" s="13">
+        <v>194.5</v>
+      </c>
+      <c r="G7" s="13"/>
+      <c r="H7" s="13" t="s">
+        <v>201</v>
+      </c>
+      <c r="I7" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="J7" s="13"/>
+      <c r="K7" s="13">
+        <v>144.9</v>
+      </c>
+      <c r="L7" s="13">
+        <v>221.4</v>
+      </c>
+      <c r="M7" s="13">
+        <v>297.5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.75">
+      <c r="A8" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="D8" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="E8" s="13">
+        <v>206</v>
+      </c>
+      <c r="F8" s="13">
+        <v>176.5</v>
+      </c>
+      <c r="G8" s="13"/>
+      <c r="H8" s="13" t="s">
+        <v>143</v>
+      </c>
+      <c r="I8" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="J8" s="13"/>
+      <c r="K8" s="13">
+        <v>130.4</v>
+      </c>
+      <c r="L8" s="13">
+        <v>206.2</v>
+      </c>
+      <c r="M8" s="13">
+        <v>280.10000000000002</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.75">
+      <c r="A9" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="B9" s="13" t="s">
+        <v>46</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>116</v>
+      </c>
+      <c r="D9" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="E9" s="13">
+        <v>247.80000305175781</v>
+      </c>
+      <c r="F9" s="13">
+        <v>232.5</v>
+      </c>
+      <c r="G9" s="13"/>
+      <c r="H9" s="13" t="s">
+        <v>261</v>
+      </c>
+      <c r="I9" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="J9" s="13"/>
+      <c r="K9" s="13">
+        <v>173.6</v>
+      </c>
+      <c r="L9" s="13">
+        <v>247.9</v>
+      </c>
+      <c r="M9" s="13">
+        <v>322.3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.75">
+      <c r="A10" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="C10" s="13" t="s">
+        <v>111</v>
+      </c>
+      <c r="D10" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="E10" s="13">
+        <v>236.8999938964844</v>
+      </c>
+      <c r="F10" s="13">
+        <v>248.5</v>
+      </c>
+      <c r="G10" s="13"/>
+      <c r="H10" s="13" t="s">
+        <v>209</v>
+      </c>
+      <c r="I10" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="J10" s="13"/>
+      <c r="K10" s="13">
+        <v>161.4</v>
+      </c>
+      <c r="L10" s="13">
+        <v>237.2</v>
+      </c>
+      <c r="M10" s="13">
+        <v>312.89999999999998</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.75">
+      <c r="A11" s="13" t="s">
+        <v>133</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>111</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="D11" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="E11" s="13">
+        <v>238.6000061035156</v>
+      </c>
+      <c r="F11" s="13">
+        <v>219.5</v>
+      </c>
+      <c r="G11" s="13"/>
+      <c r="H11" s="13" t="s">
+        <v>245</v>
+      </c>
+      <c r="I11" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="J11" s="13"/>
+      <c r="K11" s="13">
+        <v>163.80000000000001</v>
+      </c>
+      <c r="L11" s="13">
+        <v>239</v>
+      </c>
+      <c r="M11" s="13">
+        <v>313.10000000000002</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.75">
+      <c r="A12" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="B12" s="13" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>100</v>
+      </c>
+      <c r="D12" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="E12" s="13">
+        <v>246.80000305175781</v>
+      </c>
+      <c r="F12" s="13">
+        <v>241.5</v>
+      </c>
+      <c r="G12" s="13"/>
+      <c r="H12" s="13" t="s">
+        <v>244</v>
+      </c>
+      <c r="I12" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="J12" s="13"/>
+      <c r="K12" s="13">
+        <v>172.1</v>
+      </c>
+      <c r="L12" s="13">
+        <v>246.3</v>
+      </c>
+      <c r="M12" s="13">
+        <v>322.3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.75">
+      <c r="A13" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="D13" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="E13" s="13">
+        <v>240.8999938964844</v>
+      </c>
+      <c r="F13" s="13">
+        <v>230.5</v>
+      </c>
+      <c r="G13" s="13"/>
+      <c r="H13" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="I13" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="J13" s="13"/>
+      <c r="K13" s="13">
+        <v>164</v>
+      </c>
+      <c r="L13" s="13">
+        <v>240.1</v>
+      </c>
+      <c r="M13" s="13">
+        <v>316.10000000000002</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.75">
+      <c r="A14" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="B14" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="D14" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="E14" s="13">
+        <v>241.3999938964844</v>
+      </c>
+      <c r="F14" s="13">
+        <v>248.5</v>
+      </c>
+      <c r="G14" s="13"/>
+      <c r="H14" s="13" t="s">
+        <v>193</v>
+      </c>
+      <c r="I14" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="J14" s="13"/>
+      <c r="K14" s="13">
+        <v>165.4</v>
+      </c>
+      <c r="L14" s="13">
+        <v>240.3</v>
+      </c>
+      <c r="M14" s="13">
+        <v>315.5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.75">
+      <c r="A15" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="B15" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="C15" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="D15" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="E15" s="13">
+        <v>252.3999938964844</v>
+      </c>
+      <c r="F15" s="13">
+        <v>238.5</v>
+      </c>
+      <c r="G15" s="13"/>
+      <c r="H15" s="13" t="s">
+        <v>283</v>
+      </c>
+      <c r="I15" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="J15" s="13"/>
+      <c r="K15" s="13">
+        <v>175.4</v>
+      </c>
+      <c r="L15" s="13">
+        <v>252</v>
+      </c>
+      <c r="M15" s="13">
+        <v>327.7</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.75">
+      <c r="A16" s="13" t="s">
+        <v>109</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>110</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="D16" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="E16" s="13">
+        <v>232.3999938964844</v>
+      </c>
+      <c r="F16" s="13">
+        <v>222.5</v>
+      </c>
+      <c r="G16" s="13"/>
+      <c r="H16" s="13" t="s">
+        <v>214</v>
+      </c>
+      <c r="I16" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="J16" s="13"/>
+      <c r="K16" s="13">
+        <v>157.5</v>
+      </c>
+      <c r="L16" s="13">
+        <v>233.2</v>
+      </c>
+      <c r="M16" s="13">
+        <v>309.5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.75">
+      <c r="A17" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="B17" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="C17" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="D17" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="E17" s="13">
+        <v>226.8999938964844</v>
+      </c>
+      <c r="F17" s="13">
+        <v>211.5</v>
+      </c>
+      <c r="G17" s="13"/>
+      <c r="H17" s="13" t="s">
+        <v>284</v>
+      </c>
+      <c r="I17" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="J17" s="13"/>
+      <c r="K17" s="13">
+        <v>152.5</v>
+      </c>
+      <c r="L17" s="13">
+        <v>227.8</v>
+      </c>
+      <c r="M17" s="13">
+        <v>303.2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.75">
+      <c r="A18" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="B18" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="C18" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="D18" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="E18" s="13">
+        <v>251</v>
+      </c>
+      <c r="F18" s="13">
+        <v>230.5</v>
+      </c>
+      <c r="G18" s="13"/>
+      <c r="H18" s="13" t="s">
+        <v>245</v>
+      </c>
+      <c r="I18" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="J18" s="13"/>
+      <c r="K18" s="13">
+        <v>173.9</v>
+      </c>
+      <c r="L18" s="13">
+        <v>250</v>
+      </c>
+      <c r="M18" s="13">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.75">
+      <c r="A19" s="13" t="s">
+        <v>128</v>
+      </c>
+      <c r="B19" s="13" t="s">
+        <v>100</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>40</v>
+      </c>
+      <c r="D19" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="E19" s="13">
+        <v>222.8999938964844</v>
+      </c>
+      <c r="F19" s="13">
+        <v>210.5</v>
+      </c>
+      <c r="G19" s="13"/>
+      <c r="H19" s="13" t="s">
+        <v>160</v>
+      </c>
+      <c r="I19" s="21" t="s">
+        <v>19</v>
+      </c>
+      <c r="J19" s="13"/>
+      <c r="K19" s="13">
+        <v>147.9</v>
+      </c>
+      <c r="L19" s="13">
+        <v>222.3</v>
+      </c>
+      <c r="M19" s="13">
+        <v>297.5</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>